<commit_message>
chore: update specifications and parameters in master readings based on new requirements
</commit_message>
<xml_diff>
--- a/master_readings/TEST READINGS[23].xlsx
+++ b/master_readings/TEST READINGS[23].xlsx
@@ -1460,74 +1460,74 @@
       <c r="C7" s="21" t="n"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Insulation thickness (Nom.)</t>
+          <t>Insulation thickness</t>
         </is>
       </c>
       <c r="E7" s="21" t="n"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>0.35 mm</t>
+          <t>0.35 mm Min.</t>
         </is>
       </c>
       <c r="G7" s="10" t="n"/>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>0.50 mm</t>
+          <t>0.50 mm Min.</t>
         </is>
       </c>
       <c r="J7" s="10" t="n"/>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>0.60 mm</t>
+          <t>0.60 mm Min.</t>
         </is>
       </c>
       <c r="M7" s="10" t="n"/>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>0.50 mm</t>
+          <t>0.50 mm Min.</t>
         </is>
       </c>
       <c r="P7" s="10" t="n"/>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>0.30 mm</t>
+          <t>0.30 mm Min.</t>
         </is>
       </c>
       <c r="S7" s="10" t="n"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>0.30 mm</t>
+          <t>0.30 mm Min.</t>
         </is>
       </c>
       <c r="V7" s="10" t="n"/>
       <c r="X7" s="7" t="inlineStr">
         <is>
-          <t>0.30 mm</t>
+          <t>0.30 mm Min.</t>
         </is>
       </c>
       <c r="Y7" s="10" t="n"/>
       <c r="AA7" s="7" t="inlineStr">
         <is>
-          <t>0.35 mm</t>
+          <t>0.35 mm Min.</t>
         </is>
       </c>
       <c r="AB7" s="10" t="n"/>
       <c r="AD7" s="7" t="inlineStr">
         <is>
-          <t>0.50 mm</t>
+          <t>0.50 mm Min.</t>
         </is>
       </c>
       <c r="AE7" s="10" t="n"/>
       <c r="AG7" s="7" t="inlineStr">
         <is>
-          <t>0.50 mm</t>
+          <t>0.50 mm Min.</t>
         </is>
       </c>
       <c r="AH7" s="10" t="n"/>
       <c r="AJ7" s="7" t="inlineStr">
         <is>
-          <t>0.35 mm</t>
+          <t>0.35 mm Min.</t>
         </is>
       </c>
       <c r="AK7" s="10" t="n"/>
@@ -1557,19 +1557,19 @@
       <c r="AW7" s="10" t="n"/>
       <c r="AY7" s="7" t="inlineStr">
         <is>
-          <t>0.30 mm</t>
+          <t>0.30 mm Min.</t>
         </is>
       </c>
       <c r="AZ7" s="10" t="n"/>
       <c r="BB7" s="7" t="inlineStr">
         <is>
-          <t>0.24 mm</t>
+          <t>0.24 mm Min.</t>
         </is>
       </c>
       <c r="BC7" s="10" t="n"/>
       <c r="BE7" s="7" t="inlineStr">
         <is>
-          <t>0.60 mm</t>
+          <t>0.60 mm Min.</t>
         </is>
       </c>
       <c r="BF7" s="10" t="n"/>

</xml_diff>